<commit_message>
modification sort subfolders as sheet
</commit_message>
<xml_diff>
--- a/sample.xlsx
+++ b/sample.xlsx
@@ -1,28 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28324"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\TEE\02 Knowledge Sharing\excel_writer\TestEvidenceCreator\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\kokitt\git\TestEvidenceCreator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F4592F5-B3A7-41D9-BA43-2BC9E4B87D74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" tabRatio="850" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="23880" yWindow="-1665" windowWidth="29040" windowHeight="15720" tabRatio="850"/>
   </bookViews>
   <sheets>
-    <sheet name="#1" sheetId="148" r:id="rId1"/>
+    <sheet name="Final Template" sheetId="148" r:id="rId1"/>
+    <sheet name="#Preparation" sheetId="149" r:id="rId7"/>
+    <sheet name="#1" sheetId="150" r:id="rId8"/>
+    <sheet name="#2" sheetId="151" r:id="rId9"/>
+    <sheet name="#3" sheetId="152" r:id="rId10"/>
   </sheets>
   <calcPr calcId="191029"/>
   <customWorkbookViews>
-    <customWorkbookView name="桑木 大輔 - Personal View" guid="{686D9949-37D0-401E-BF09-C298B84DC1DD}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1920" windowHeight="855" tabRatio="674" activeSheetId="4"/>
-    <customWorkbookView name="莫 瑞琳/DIR Global Service Support Dept. - 個人用ビュー" guid="{F9AEA311-B555-4CE8-8AFE-56E0C40CE68C}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1916" windowHeight="850" tabRatio="916" activeSheetId="6"/>
-    <customWorkbookView name="Daisuke Kuwagi/DIR Global Service Support Dept. - 個人用ビュー" guid="{47A13601-03B4-449A-8A5A-67581A7123F4}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1916" windowHeight="849" tabRatio="916" activeSheetId="10"/>
-    <customWorkbookView name="kanrisya - 個人用ビュー" guid="{69F5E423-CBB8-40ED-8D62-CF605B63DF1D}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1362" windowHeight="538" tabRatio="916" activeSheetId="6"/>
-    <customWorkbookView name="Kazuki Ogiya/DIR Global Service Support Dept. - 個人用ビュー" guid="{676A5308-DD69-4B23-A2F4-B4BDED89FB27}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1916" windowHeight="850" tabRatio="916" activeSheetId="6" showComments="commIndAndComment"/>
-    <customWorkbookView name="Tomoko Uwatoko/DIR Global Service Support Dept. - 個人用ビュー" guid="{181D197A-1D89-4CFD-8223-28B687C6926D}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1916" windowHeight="778" tabRatio="916" activeSheetId="2"/>
+    <customWorkbookView activeSheetId="4" guid="{686D9949-37D0-401E-BF09-C298B84DC1DD}" maximized="true" mergeInterval="0" name="桑木 大輔 - Personal View" personalView="true" tabRatio="674" windowHeight="855" windowWidth="1920"/>
+    <customWorkbookView activeSheetId="6" guid="{F9AEA311-B555-4CE8-8AFE-56E0C40CE68C}" maximized="true" mergeInterval="0" name="莫 瑞琳/DIR Global Service Support Dept. - 個人用ビュー" personalView="true" tabRatio="916" windowHeight="850" windowWidth="1916"/>
+    <customWorkbookView activeSheetId="10" guid="{47A13601-03B4-449A-8A5A-67581A7123F4}" maximized="true" mergeInterval="0" name="Daisuke Kuwagi/DIR Global Service Support Dept. - 個人用ビュー" personalView="true" tabRatio="916" windowHeight="849" windowWidth="1916"/>
+    <customWorkbookView activeSheetId="6" guid="{69F5E423-CBB8-40ED-8D62-CF605B63DF1D}" maximized="true" mergeInterval="0" name="kanrisya - 個人用ビュー" personalView="true" tabRatio="916" windowHeight="538" windowWidth="1362"/>
+    <customWorkbookView activeSheetId="6" guid="{676A5308-DD69-4B23-A2F4-B4BDED89FB27}" maximized="true" mergeInterval="0" name="Kazuki Ogiya/DIR Global Service Support Dept. - 個人用ビュー" personalView="true" showComments="commIndAndComment" tabRatio="916" windowHeight="850" windowWidth="1916"/>
+    <customWorkbookView activeSheetId="2" guid="{181D197A-1D89-4CFD-8223-28B687C6926D}" maximized="true" mergeInterval="0" name="Tomoko Uwatoko/DIR Global Service Support Dept. - 個人用ビュー" personalView="true" tabRatio="916" windowHeight="778" windowWidth="1916"/>
   </customWorkbookViews>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -41,7 +44,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ap="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:op="http://schemas.openxmlformats.org/officeDocument/2006/custom-properties" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing" xmlns:comp="http://schemas.openxmlformats.org/drawingml/2006/compatibility" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:lc="http://schemas.openxmlformats.org/drawingml/2006/lockedCanvas" xmlns:pic="http://schemas.openxmlformats.org/drawingml/2006/picture" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:sl="http://schemas.openxmlformats.org/schemaLibrary/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xne="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mso="http://schemas.microsoft.com/office/2006/01/customui" xmlns:ax="http://schemas.microsoft.com/office/2006/activeX" xmlns:cppr="http://schemas.microsoft.com/office/2006/coverPageProps" xmlns:cdip="http://schemas.microsoft.com/office/2006/customDocumentInformationPanel" xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ntns="http://schemas.microsoft.com/office/2006/metadata/customXsn" xmlns:lp="http://schemas.microsoft.com/office/2006/metadata/longProperties" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" xmlns:msink="http://schemas.microsoft.com/ink/2010/main" xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" xmlns:cdr14="http://schemas.microsoft.com/office/drawing/2010/chartDrawing" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns:pic14="http://schemas.microsoft.com/office/drawing/2010/picture" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:dsp="http://schemas.microsoft.com/office/drawing/2008/diagram" xmlns:mso14="http://schemas.microsoft.com/office/2009/07/customui" xmlns:dgm14="http://schemas.microsoft.com/office/drawing/2010/diagram" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:xr4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision4" xmlns:xr5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision5" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr7="http://schemas.microsoft.com/office/spreadsheetml/2016/revision7" xmlns:xr8="http://schemas.microsoft.com/office/spreadsheetml/2016/revision8" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr11="http://schemas.microsoft.com/office/spreadsheetml/2016/revision11" xmlns:xr12="http://schemas.microsoft.com/office/spreadsheetml/2016/revision12" xmlns:xr13="http://schemas.microsoft.com/office/spreadsheetml/2016/revision13" xmlns:xr14="http://schemas.microsoft.com/office/spreadsheetml/2016/revision14" xmlns:xr15="http://schemas.microsoft.com/office/spreadsheetml/2016/revision15" xmlns:x16="http://schemas.microsoft.com/office/spreadsheetml/2014/11/main" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:mo="http://schemas.microsoft.com/office/mac/office/2008/main" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:o="urn:schemas-microsoft-com:office:office" xmlns:v="urn:schemas-microsoft-com:vml" mc:Ignorable="c14 cdr14 a14 pic14 x14 xdr14 x14ac dsp mso14 dgm14 x15 x12ac x15ac xr xr2 xr3 xr4 xr5 xr6 xr7 xr8 xr9 xr10 xr11 xr12 xr13 xr14 xr15 x15 x16 x16r2 mo mx mv o v" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="#,##0;\-#,##0;&quot;-&quot;"/>
     <numFmt numFmtId="165" formatCode="[$-409]d\-mmm\-yy;@"/>
@@ -80,7 +83,7 @@
       <family val="2"/>
     </font>
     <font>
-      <b/>
+      <b val="1"/>
       <sz val="12"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -119,7 +122,7 @@
       <charset val="128"/>
     </font>
     <font>
-      <b/>
+      <b val="1"/>
       <sz val="18"/>
       <color indexed="56"/>
       <name val="ＭＳ Ｐゴシック"/>
@@ -127,7 +130,7 @@
       <charset val="128"/>
     </font>
     <font>
-      <b/>
+      <b val="1"/>
       <sz val="11"/>
       <color indexed="9"/>
       <name val="ＭＳ ゴシック"/>
@@ -156,7 +159,7 @@
       <charset val="128"/>
     </font>
     <font>
-      <b/>
+      <b val="1"/>
       <sz val="11"/>
       <color indexed="63"/>
       <name val="ＭＳ ゴシック"/>
@@ -178,7 +181,7 @@
       <charset val="128"/>
     </font>
     <font>
-      <b/>
+      <b val="1"/>
       <sz val="15"/>
       <color indexed="56"/>
       <name val="ＭＳ ゴシック"/>
@@ -186,7 +189,7 @@
       <charset val="128"/>
     </font>
     <font>
-      <b/>
+      <b val="1"/>
       <sz val="13"/>
       <color indexed="56"/>
       <name val="ＭＳ ゴシック"/>
@@ -194,7 +197,7 @@
       <charset val="128"/>
     </font>
     <font>
-      <b/>
+      <b val="1"/>
       <sz val="11"/>
       <color indexed="56"/>
       <name val="ＭＳ ゴシック"/>
@@ -202,7 +205,7 @@
       <charset val="128"/>
     </font>
     <font>
-      <b/>
+      <b val="1"/>
       <sz val="11"/>
       <color indexed="52"/>
       <name val="ＭＳ ゴシック"/>
@@ -210,7 +213,7 @@
       <charset val="128"/>
     </font>
     <font>
-      <i/>
+      <i val="1"/>
       <sz val="11"/>
       <color indexed="23"/>
       <name val="ＭＳ ゴシック"/>
@@ -225,7 +228,7 @@
       <charset val="128"/>
     </font>
     <font>
-      <b/>
+      <b val="1"/>
       <sz val="11"/>
       <color indexed="8"/>
       <name val="ＭＳ ゴシック"/>
@@ -526,26 +529,26 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="38" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="38" fontId="3" fillId="0" borderId="0" applyFont="false" applyFill="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyFill="false" applyBorder="false" applyAlignment="false"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyNumberFormat="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="false" applyFill="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="false" applyFont="false" applyFill="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment vertical="top"/>
-      <protection locked="0"/>
+      <protection locked="false"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="38" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="38" fontId="2" fillId="0" borderId="0" applyFont="false" applyFill="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0">
@@ -554,130 +557,130 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="12" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="13" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="14" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="15" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="20" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="22" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="23" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="23" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="16" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="17" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="18" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="13" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="14" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="19" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="false" applyFill="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="20" borderId="3" applyNumberFormat="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="21" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="22" borderId="4" applyNumberFormat="false" applyFont="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" applyNumberFormat="false" applyFill="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="6" applyNumberFormat="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="23" borderId="7" applyNumberFormat="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" applyNumberFormat="false" applyFill="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="9" applyNumberFormat="false" applyFill="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" applyNumberFormat="false" applyFill="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="false" applyFill="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="23" borderId="6" applyNumberFormat="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyNumberFormat="false" applyFill="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="false" applyFill="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="11" applyNumberFormat="false" applyFill="false" applyAlignment="false" applyProtection="false">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0"/>
@@ -699,80 +702,80 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="24" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="24" borderId="0" xfId="0" applyFill="true"/>
   </cellXfs>
   <cellStyles count="68">
-    <cellStyle name="_x000d__x000a_JournalTemplate=C:\COMFO\CTALK\JOURSTD.TPL_x000d__x000a_LbStateAddress=3 3 0 251 1 89 2 311_x000d__x000a_LbStateJou" xfId="58" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
-    <cellStyle name="??_(????)??????" xfId="59" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
-    <cellStyle name="0,0_x000d__x000a_NA_x000d__x000a_" xfId="2" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
-    <cellStyle name="20% - アクセント 1" xfId="14" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
-    <cellStyle name="20% - アクセント 2" xfId="15" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
-    <cellStyle name="20% - アクセント 3" xfId="16" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
-    <cellStyle name="20% - アクセント 4" xfId="17" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
-    <cellStyle name="20% - アクセント 5" xfId="18" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
-    <cellStyle name="20% - アクセント 6" xfId="19" xr:uid="{00000000-0005-0000-0000-000008000000}"/>
-    <cellStyle name="40% - アクセント 1" xfId="20" xr:uid="{00000000-0005-0000-0000-000009000000}"/>
-    <cellStyle name="40% - アクセント 2" xfId="21" xr:uid="{00000000-0005-0000-0000-00000A000000}"/>
-    <cellStyle name="40% - アクセント 3" xfId="22" xr:uid="{00000000-0005-0000-0000-00000B000000}"/>
-    <cellStyle name="40% - アクセント 4" xfId="23" xr:uid="{00000000-0005-0000-0000-00000C000000}"/>
-    <cellStyle name="40% - アクセント 5" xfId="24" xr:uid="{00000000-0005-0000-0000-00000D000000}"/>
-    <cellStyle name="40% - アクセント 6" xfId="25" xr:uid="{00000000-0005-0000-0000-00000E000000}"/>
-    <cellStyle name="60% - アクセント 1" xfId="26" xr:uid="{00000000-0005-0000-0000-00000F000000}"/>
-    <cellStyle name="60% - アクセント 2" xfId="27" xr:uid="{00000000-0005-0000-0000-000010000000}"/>
-    <cellStyle name="60% - アクセント 3" xfId="28" xr:uid="{00000000-0005-0000-0000-000011000000}"/>
-    <cellStyle name="60% - アクセント 4" xfId="29" xr:uid="{00000000-0005-0000-0000-000012000000}"/>
-    <cellStyle name="60% - アクセント 5" xfId="30" xr:uid="{00000000-0005-0000-0000-000013000000}"/>
-    <cellStyle name="60% - アクセント 6" xfId="31" xr:uid="{00000000-0005-0000-0000-000014000000}"/>
-    <cellStyle name="Calc Currency (0)" xfId="4" xr:uid="{00000000-0005-0000-0000-000015000000}"/>
-    <cellStyle name="Comma [0] 2" xfId="3" xr:uid="{00000000-0005-0000-0000-000016000000}"/>
-    <cellStyle name="Header1" xfId="5" xr:uid="{00000000-0005-0000-0000-000017000000}"/>
-    <cellStyle name="Header2" xfId="6" xr:uid="{00000000-0005-0000-0000-000018000000}"/>
+    <cellStyle name="_x000d__x000a_JournalTemplate=C:\COMFO\CTALK\JOURSTD.TPL_x000d__x000a_LbStateAddress=3 3 0 251 1 89 2 311_x000d__x000a_LbStateJou" xfId="58"/>
+    <cellStyle name="??_(????)??????" xfId="59"/>
+    <cellStyle name="0,0_x000d__x000a_NA_x000d__x000a_" xfId="2"/>
+    <cellStyle name="20% - アクセント 1" xfId="14"/>
+    <cellStyle name="20% - アクセント 2" xfId="15"/>
+    <cellStyle name="20% - アクセント 3" xfId="16"/>
+    <cellStyle name="20% - アクセント 4" xfId="17"/>
+    <cellStyle name="20% - アクセント 5" xfId="18"/>
+    <cellStyle name="20% - アクセント 6" xfId="19"/>
+    <cellStyle name="40% - アクセント 1" xfId="20"/>
+    <cellStyle name="40% - アクセント 2" xfId="21"/>
+    <cellStyle name="40% - アクセント 3" xfId="22"/>
+    <cellStyle name="40% - アクセント 4" xfId="23"/>
+    <cellStyle name="40% - アクセント 5" xfId="24"/>
+    <cellStyle name="40% - アクセント 6" xfId="25"/>
+    <cellStyle name="60% - アクセント 1" xfId="26"/>
+    <cellStyle name="60% - アクセント 2" xfId="27"/>
+    <cellStyle name="60% - アクセント 3" xfId="28"/>
+    <cellStyle name="60% - アクセント 4" xfId="29"/>
+    <cellStyle name="60% - アクセント 5" xfId="30"/>
+    <cellStyle name="60% - アクセント 6" xfId="31"/>
+    <cellStyle name="Calc Currency (0)" xfId="4"/>
+    <cellStyle name="Comma [0] 2" xfId="3"/>
+    <cellStyle name="Header1" xfId="5"/>
+    <cellStyle name="Header2" xfId="6"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="7" xr:uid="{00000000-0005-0000-0000-00001A000000}"/>
-    <cellStyle name="Normal 2 2" xfId="60" xr:uid="{00000000-0005-0000-0000-00001B000000}"/>
-    <cellStyle name="Normal 2 3" xfId="61" xr:uid="{00000000-0005-0000-0000-00001C000000}"/>
-    <cellStyle name="Normal 2 4" xfId="62" xr:uid="{00000000-0005-0000-0000-00001D000000}"/>
-    <cellStyle name="Normal 3" xfId="32" xr:uid="{00000000-0005-0000-0000-00001E000000}"/>
-    <cellStyle name="Normal 3 2" xfId="63" xr:uid="{00000000-0005-0000-0000-00001F000000}"/>
-    <cellStyle name="Normal 4" xfId="33" xr:uid="{00000000-0005-0000-0000-000020000000}"/>
-    <cellStyle name="Normal 4 2" xfId="64" xr:uid="{00000000-0005-0000-0000-000021000000}"/>
-    <cellStyle name="Normal 5" xfId="34" xr:uid="{00000000-0005-0000-0000-000022000000}"/>
-    <cellStyle name="Normal 5 2" xfId="65" xr:uid="{00000000-0005-0000-0000-000023000000}"/>
-    <cellStyle name="Normal 6" xfId="66" xr:uid="{00000000-0005-0000-0000-000024000000}"/>
-    <cellStyle name="アクセント 1" xfId="35" xr:uid="{00000000-0005-0000-0000-000025000000}"/>
-    <cellStyle name="アクセント 2" xfId="36" xr:uid="{00000000-0005-0000-0000-000026000000}"/>
-    <cellStyle name="アクセント 3" xfId="37" xr:uid="{00000000-0005-0000-0000-000027000000}"/>
-    <cellStyle name="アクセント 4" xfId="38" xr:uid="{00000000-0005-0000-0000-000028000000}"/>
-    <cellStyle name="アクセント 5" xfId="39" xr:uid="{00000000-0005-0000-0000-000029000000}"/>
-    <cellStyle name="アクセント 6" xfId="40" xr:uid="{00000000-0005-0000-0000-00002A000000}"/>
-    <cellStyle name="タイトル" xfId="41" xr:uid="{00000000-0005-0000-0000-00002B000000}"/>
-    <cellStyle name="チェック セル" xfId="42" xr:uid="{00000000-0005-0000-0000-00002C000000}"/>
-    <cellStyle name="どちらでもない" xfId="43" xr:uid="{00000000-0005-0000-0000-00002D000000}"/>
-    <cellStyle name="パーセント 2" xfId="8" xr:uid="{00000000-0005-0000-0000-00002E000000}"/>
-    <cellStyle name="ハイパーリンク 2" xfId="9" xr:uid="{00000000-0005-0000-0000-00002F000000}"/>
-    <cellStyle name="メモ" xfId="44" xr:uid="{00000000-0005-0000-0000-000030000000}"/>
-    <cellStyle name="リンク セル" xfId="45" xr:uid="{00000000-0005-0000-0000-000031000000}"/>
-    <cellStyle name="표준_(정보부문)월별인원계획" xfId="67" xr:uid="{00000000-0005-0000-0000-000032000000}"/>
-    <cellStyle name="入力" xfId="46" xr:uid="{00000000-0005-0000-0000-000033000000}"/>
-    <cellStyle name="出力" xfId="47" xr:uid="{00000000-0005-0000-0000-000034000000}"/>
-    <cellStyle name="悪い" xfId="48" xr:uid="{00000000-0005-0000-0000-000035000000}"/>
-    <cellStyle name="未定義" xfId="10" xr:uid="{00000000-0005-0000-0000-000036000000}"/>
-    <cellStyle name="桁区切り 2" xfId="11" xr:uid="{00000000-0005-0000-0000-000037000000}"/>
-    <cellStyle name="標準 2" xfId="12" xr:uid="{00000000-0005-0000-0000-000038000000}"/>
-    <cellStyle name="標準 3" xfId="13" xr:uid="{00000000-0005-0000-0000-000039000000}"/>
-    <cellStyle name="標準_02_UT完了報告書_タスク管理_20120314_試験完了" xfId="1" xr:uid="{00000000-0005-0000-0000-00003A000000}"/>
-    <cellStyle name="良い" xfId="49" xr:uid="{00000000-0005-0000-0000-00003B000000}"/>
-    <cellStyle name="見出し 1" xfId="50" xr:uid="{00000000-0005-0000-0000-00003C000000}"/>
-    <cellStyle name="見出し 2" xfId="51" xr:uid="{00000000-0005-0000-0000-00003D000000}"/>
-    <cellStyle name="見出し 3" xfId="52" xr:uid="{00000000-0005-0000-0000-00003E000000}"/>
-    <cellStyle name="見出し 4" xfId="53" xr:uid="{00000000-0005-0000-0000-00003F000000}"/>
-    <cellStyle name="計算" xfId="54" xr:uid="{00000000-0005-0000-0000-000040000000}"/>
-    <cellStyle name="説明文" xfId="55" xr:uid="{00000000-0005-0000-0000-000041000000}"/>
-    <cellStyle name="警告文" xfId="56" xr:uid="{00000000-0005-0000-0000-000042000000}"/>
-    <cellStyle name="集計" xfId="57" xr:uid="{00000000-0005-0000-0000-000043000000}"/>
+    <cellStyle name="Normal 2" xfId="7"/>
+    <cellStyle name="Normal 2 2" xfId="60"/>
+    <cellStyle name="Normal 2 3" xfId="61"/>
+    <cellStyle name="Normal 2 4" xfId="62"/>
+    <cellStyle name="Normal 3" xfId="32"/>
+    <cellStyle name="Normal 3 2" xfId="63"/>
+    <cellStyle name="Normal 4" xfId="33"/>
+    <cellStyle name="Normal 4 2" xfId="64"/>
+    <cellStyle name="Normal 5" xfId="34"/>
+    <cellStyle name="Normal 5 2" xfId="65"/>
+    <cellStyle name="Normal 6" xfId="66"/>
+    <cellStyle name="アクセント 1" xfId="35"/>
+    <cellStyle name="アクセント 2" xfId="36"/>
+    <cellStyle name="アクセント 3" xfId="37"/>
+    <cellStyle name="アクセント 4" xfId="38"/>
+    <cellStyle name="アクセント 5" xfId="39"/>
+    <cellStyle name="アクセント 6" xfId="40"/>
+    <cellStyle name="タイトル" xfId="41"/>
+    <cellStyle name="チェック セル" xfId="42"/>
+    <cellStyle name="どちらでもない" xfId="43"/>
+    <cellStyle name="パーセント 2" xfId="8"/>
+    <cellStyle name="ハイパーリンク 2" xfId="9"/>
+    <cellStyle name="メモ" xfId="44"/>
+    <cellStyle name="リンク セル" xfId="45"/>
+    <cellStyle name="표준_(정보부문)월별인원계획" xfId="67"/>
+    <cellStyle name="入力" xfId="46"/>
+    <cellStyle name="出力" xfId="47"/>
+    <cellStyle name="悪い" xfId="48"/>
+    <cellStyle name="未定義" xfId="10"/>
+    <cellStyle name="桁区切り 2" xfId="11"/>
+    <cellStyle name="標準 2" xfId="12"/>
+    <cellStyle name="標準 3" xfId="13"/>
+    <cellStyle name="標準_02_UT完了報告書_タスク管理_20120314_試験完了" xfId="1"/>
+    <cellStyle name="良い" xfId="49"/>
+    <cellStyle name="見出し 1" xfId="50"/>
+    <cellStyle name="見出し 2" xfId="51"/>
+    <cellStyle name="見出し 3" xfId="52"/>
+    <cellStyle name="見出し 4" xfId="53"/>
+    <cellStyle name="計算" xfId="54"/>
+    <cellStyle name="説明文" xfId="55"/>
+    <cellStyle name="警告文" xfId="56"/>
+    <cellStyle name="集計" xfId="57"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultPivotStyle="PivotStyleLight16" defaultTableStyle="TableStyleMedium2"/>
   <colors>
     <mruColors>
       <color rgb="FFFF7C80"/>
@@ -792,8 +795,768 @@
 </styleSheet>
 </file>
 
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>35</xdr:col>
+      <xdr:colOff>257175</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 2" descr=""/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="false"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect"/>
+        <a:ln/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>38</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>72</xdr:col>
+      <xdr:colOff>257175</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 3" descr=""/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="false"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect"/>
+        <a:ln/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>75</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>109</xdr:col>
+      <xdr:colOff>257175</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 4" descr=""/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="false"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect"/>
+        <a:ln/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>112</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>146</xdr:col>
+      <xdr:colOff>257175</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 5" descr=""/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="false"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect"/>
+        <a:ln/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>149</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>183</xdr:col>
+      <xdr:colOff>257175</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Picture 6" descr=""/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="false"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect"/>
+        <a:ln/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>35</xdr:col>
+      <xdr:colOff>257175</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 2" descr=""/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="false"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect"/>
+        <a:ln/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>38</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>72</xdr:col>
+      <xdr:colOff>257175</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 3" descr=""/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="false"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect"/>
+        <a:ln/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>75</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>109</xdr:col>
+      <xdr:colOff>257175</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 4" descr=""/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="false"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect"/>
+        <a:ln/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>112</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>146</xdr:col>
+      <xdr:colOff>257175</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 5" descr=""/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="false"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect"/>
+        <a:ln/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>149</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>183</xdr:col>
+      <xdr:colOff>257175</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Picture 6" descr=""/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="false"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect"/>
+        <a:ln/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>35</xdr:col>
+      <xdr:colOff>257175</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 2" descr=""/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="false"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect"/>
+        <a:ln/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>38</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>72</xdr:col>
+      <xdr:colOff>257175</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 3" descr=""/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="false"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect"/>
+        <a:ln/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>75</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>109</xdr:col>
+      <xdr:colOff>257175</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 4" descr=""/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="false"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect"/>
+        <a:ln/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>112</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>146</xdr:col>
+      <xdr:colOff>257175</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 5" descr=""/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="false"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect"/>
+        <a:ln/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>149</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>183</xdr:col>
+      <xdr:colOff>257175</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Picture 6" descr=""/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="false"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect"/>
+        <a:ln/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>35</xdr:col>
+      <xdr:colOff>257175</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 2" descr=""/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="false"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect"/>
+        <a:ln/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>38</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>72</xdr:col>
+      <xdr:colOff>257175</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 3" descr=""/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="false"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect"/>
+        <a:ln/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>75</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>109</xdr:col>
+      <xdr:colOff>257175</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 4" descr=""/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="false"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect"/>
+        <a:ln/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>112</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>146</xdr:col>
+      <xdr:colOff>257175</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 5" descr=""/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="false"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect"/>
+        <a:ln/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>149</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>183</xdr:col>
+      <xdr:colOff>257175</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Picture 6" descr=""/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="false"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect"/>
+        <a:ln/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1056,46 +1819,174 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{413A1042-015E-4BEA-B464-50B5CF99346E}">
   <sheetPr codeName="Sheet5">
-    <pageSetUpPr fitToPage="1"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1"/>
   <sheetFormatPr defaultColWidth="3.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="3.7109375" customWidth="1"/>
+    <col customWidth="true" max="1" min="1" width="3.7109375"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="8.25" customHeight="1">
+    <row r="1" spans="1:1" ht="8.25" customHeight="true">
       <c r="A1" s="1"/>
     </row>
   </sheetData>
-  <printOptions horizontalCentered="1"/>
+  <printOptions horizontalCentered="true"/>
   <pageMargins left="0.3" right="0.3" top="0.3" bottom="0.3" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" fitToWidth="0" orientation="landscape" r:id="rId1"/>
+  <pageSetup fitToHeight="1" fitToWidth="0" r:id="rId1" orientation="landscape" paperSize="9"/>
   <rowBreaks count="1" manualBreakCount="1">
-    <brk id="39" max="16383" man="1"/>
+    <brk id="39" max="16383" man="true"/>
   </rowBreaks>
   <colBreaks count="20" manualBreakCount="20">
-    <brk id="37" max="1048575" man="1"/>
-    <brk id="74" max="1048575" man="1"/>
-    <brk id="111" max="1048575" man="1"/>
-    <brk id="148" max="1048575" man="1"/>
-    <brk id="185" max="1048575" man="1"/>
-    <brk id="222" max="37" man="1"/>
-    <brk id="259" max="1048575" man="1"/>
-    <brk id="296" max="1048575" man="1"/>
-    <brk id="333" max="37" man="1"/>
-    <brk id="333" max="1048575" man="1"/>
-    <brk id="370" max="1048575" man="1"/>
-    <brk id="407" max="1048575" man="1"/>
-    <brk id="444" max="1048575" man="1"/>
-    <brk id="481" max="1048575" man="1"/>
-    <brk id="518" max="1048575" man="1"/>
-    <brk id="555" max="1048575" man="1"/>
-    <brk id="592" max="1048575" man="1"/>
-    <brk id="629" max="1048575" man="1"/>
-    <brk id="666" max="1048575" man="1"/>
-    <brk id="703" max="1048575" man="1"/>
+    <brk id="37" max="1048575" man="true"/>
+    <brk id="74" max="1048575" man="true"/>
+    <brk id="111" max="1048575" man="true"/>
+    <brk id="148" max="1048575" man="true"/>
+    <brk id="185" max="1048575" man="true"/>
+    <brk id="222" max="37" man="true"/>
+    <brk id="259" max="1048575" man="true"/>
+    <brk id="296" max="1048575" man="true"/>
+    <brk id="333" max="37" man="true"/>
+    <brk id="333" max="1048575" man="true"/>
+    <brk id="370" max="1048575" man="true"/>
+    <brk id="407" max="1048575" man="true"/>
+    <brk id="444" max="1048575" man="true"/>
+    <brk id="481" max="1048575" man="true"/>
+    <brk id="518" max="1048575" man="true"/>
+    <brk id="555" max="1048575" man="true"/>
+    <brk id="592" max="1048575" man="true"/>
+    <brk id="629" max="1048575" man="true"/>
+    <brk id="666" max="1048575" man="true"/>
+    <brk id="703" max="1048575" man="true"/>
   </colBreaks>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet149.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{413A1042-015E-4BEA-B464-50B5CF99346E}">
+  <sheetPr codeName="Sheet5">
+    <pageSetUpPr fitToPage="true"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="3.7109375" defaultRowHeight="15"/>
+  <cols>
+    <col customWidth="true" max="1" min="1" width="3.7109375"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" ht="8.25" customHeight="true">
+      <c r="A1" s="1"/>
+    </row>
+  </sheetData>
+  <printOptions horizontalCentered="true"/>
+  <pageMargins left="0.3" right="0.3" top="0.3" bottom="0.3" header="0.3" footer="0.3"/>
+  <pageSetup fitToHeight="1" fitToWidth="0" orientation="landscape" paperSize="9"/>
+  <rowBreaks count="1" manualBreakCount="1">
+    <brk id="39" max="16383" man="true"/>
+  </rowBreaks>
+  <colBreaks count="5" manualBreakCount="5">
+    <brk id="37" max="1048575" man="true"/>
+    <brk id="74" max="1048575" man="true"/>
+    <brk id="111" max="1048575" man="true"/>
+    <brk id="148" max="1048575" man="true"/>
+    <brk id="185" max="1048575" man="true"/>
+  </colBreaks>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet150.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{413A1042-015E-4BEA-B464-50B5CF99346E}">
+  <sheetPr codeName="Sheet5">
+    <pageSetUpPr fitToPage="true"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="3.7109375" defaultRowHeight="15"/>
+  <cols>
+    <col customWidth="true" max="1" min="1" width="3.7109375"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" ht="8.25" customHeight="true">
+      <c r="A1" s="1"/>
+    </row>
+  </sheetData>
+  <printOptions horizontalCentered="true"/>
+  <pageMargins left="0.3" right="0.3" top="0.3" bottom="0.3" header="0.3" footer="0.3"/>
+  <pageSetup fitToHeight="1" fitToWidth="0" orientation="landscape" paperSize="9"/>
+  <rowBreaks count="1" manualBreakCount="1">
+    <brk id="39" max="16383" man="true"/>
+  </rowBreaks>
+  <colBreaks count="5" manualBreakCount="5">
+    <brk id="37" max="1048575" man="true"/>
+    <brk id="74" max="1048575" man="true"/>
+    <brk id="111" max="1048575" man="true"/>
+    <brk id="148" max="1048575" man="true"/>
+    <brk id="185" max="1048575" man="true"/>
+  </colBreaks>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet151.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{413A1042-015E-4BEA-B464-50B5CF99346E}">
+  <sheetPr codeName="Sheet5">
+    <pageSetUpPr fitToPage="true"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="3.7109375" defaultRowHeight="15"/>
+  <cols>
+    <col customWidth="true" max="1" min="1" width="3.7109375"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" ht="8.25" customHeight="true">
+      <c r="A1" s="1"/>
+    </row>
+  </sheetData>
+  <printOptions horizontalCentered="true"/>
+  <pageMargins left="0.3" right="0.3" top="0.3" bottom="0.3" header="0.3" footer="0.3"/>
+  <pageSetup fitToHeight="1" fitToWidth="0" orientation="landscape" paperSize="9"/>
+  <rowBreaks count="1" manualBreakCount="1">
+    <brk id="39" max="16383" man="true"/>
+  </rowBreaks>
+  <colBreaks count="5" manualBreakCount="5">
+    <brk id="37" max="1048575" man="true"/>
+    <brk id="74" max="1048575" man="true"/>
+    <brk id="111" max="1048575" man="true"/>
+    <brk id="148" max="1048575" man="true"/>
+    <brk id="185" max="1048575" man="true"/>
+  </colBreaks>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet152.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{413A1042-015E-4BEA-B464-50B5CF99346E}">
+  <sheetPr codeName="Sheet5">
+    <pageSetUpPr fitToPage="true"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="3.7109375" defaultRowHeight="15"/>
+  <cols>
+    <col customWidth="true" max="1" min="1" width="3.7109375"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" ht="8.25" customHeight="true">
+      <c r="A1" s="1"/>
+    </row>
+  </sheetData>
+  <printOptions horizontalCentered="true"/>
+  <pageMargins left="0.3" right="0.3" top="0.3" bottom="0.3" header="0.3" footer="0.3"/>
+  <pageSetup fitToHeight="1" fitToWidth="0" orientation="landscape" paperSize="9"/>
+  <rowBreaks count="1" manualBreakCount="1">
+    <brk id="39" max="16383" man="true"/>
+  </rowBreaks>
+  <colBreaks count="5" manualBreakCount="5">
+    <brk id="37" max="1048575" man="true"/>
+    <brk id="74" max="1048575" man="true"/>
+    <brk id="111" max="1048575" man="true"/>
+    <brk id="148" max="1048575" man="true"/>
+    <brk id="185" max="1048575" man="true"/>
+  </colBreaks>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>